<commit_message>
calc_type_1 created for handling corp zero coupon and fixed
</commit_message>
<xml_diff>
--- a/datos_y_modelos/Domestic/domestic_sovereign_curve_brazil.xlsx
+++ b/datos_y_modelos/Domestic/domestic_sovereign_curve_brazil.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bloomberglp-my.sharepoint.com/personal/tsiqueira4_bloomberg_com/Documents/Desktop/master_thesis_economics/datos_y_modelos/Domestic/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{7055E1ED-3CA2-421B-B298-A516ACF4BB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5013B82-16D6-4C73-8F83-0461F19DD3DC}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="8_{7055E1ED-3CA2-421B-B298-A516ACF4BB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{375C73F9-BFA6-4C56-84F1-682F03E38D81}"/>
   <bookViews>
     <workbookView xWindow="-70" yWindow="10690" windowWidth="19420" windowHeight="11620" xr2:uid="{4FA8D609-CF7D-453F-9379-B1555420C1B0}"/>
   </bookViews>
@@ -2678,7 +2678,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A970A97D-4899-4477-842A-DD8D42C7E015}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2785,11 +2784,11 @@
       </c>
       <c r="M2">
         <f t="shared" ref="M2:M48" ca="1" si="0">D2-$R$2</f>
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="N2" s="3">
         <f ca="1">M2/365</f>
-        <v>3.287671232876712E-2</v>
+        <v>1.9178082191780823E-2</v>
       </c>
       <c r="O2" t="str">
         <f ca="1">IF(N2&gt;36,"&gt;36y",ROUND(N2,0)&amp;"y")</f>
@@ -2803,10 +2802,10 @@
       </c>
       <c r="R2" s="2">
         <f ca="1">TODAY()</f>
-        <v>45827</v>
+        <v>45832</v>
       </c>
     </row>
-    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2845,11 +2844,11 @@
       </c>
       <c r="M3">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N3" s="3">
         <f t="shared" ref="N3:N48" ca="1" si="1">M3/365</f>
-        <v>0.20273972602739726</v>
+        <v>0.18904109589041096</v>
       </c>
       <c r="O3" t="str">
         <f t="shared" ref="O3:O48" ca="1" si="2">IF(N3&gt;36,"&gt;36y",ROUND(N3,0)&amp;"y")</f>
@@ -2892,11 +2891,11 @@
       </c>
       <c r="M4">
         <f t="shared" ca="1" si="0"/>
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="N4" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.28493150684931506</v>
+        <v>0.27123287671232876</v>
       </c>
       <c r="O4" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -2942,11 +2941,11 @@
       </c>
       <c r="M5">
         <f t="shared" ca="1" si="0"/>
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="N5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.53698630136986303</v>
+        <v>0.52328767123287667</v>
       </c>
       <c r="O5" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -2959,7 +2958,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2998,11 +2997,11 @@
       </c>
       <c r="M6">
         <f t="shared" ca="1" si="0"/>
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="N6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.69863013698630139</v>
+        <v>0.68493150684931503</v>
       </c>
       <c r="O6" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3045,11 +3044,11 @@
       </c>
       <c r="M7">
         <f t="shared" ca="1" si="0"/>
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="N7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>0.78356164383561644</v>
+        <v>0.76986301369863008</v>
       </c>
       <c r="O7" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3095,11 +3094,11 @@
       </c>
       <c r="M8">
         <f t="shared" ca="1" si="0"/>
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="N8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.0328767123287672</v>
+        <v>1.0191780821917809</v>
       </c>
       <c r="O8" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3112,7 +3111,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -3151,11 +3150,11 @@
       </c>
       <c r="M9">
         <f t="shared" ca="1" si="0"/>
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="N9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.1561643835616437</v>
+        <v>1.1424657534246576</v>
       </c>
       <c r="O9" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3165,7 +3164,7 @@
         <v>4436.9474769999997</v>
       </c>
     </row>
-    <row r="10" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -3204,11 +3203,11 @@
       </c>
       <c r="M10">
         <f t="shared" ca="1" si="0"/>
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="N10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.2027397260273973</v>
+        <v>1.189041095890411</v>
       </c>
       <c r="O10" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3251,11 +3250,11 @@
       </c>
       <c r="M11">
         <f t="shared" ca="1" si="0"/>
-        <v>469</v>
+        <v>464</v>
       </c>
       <c r="N11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.284931506849315</v>
+        <v>1.2712328767123289</v>
       </c>
       <c r="O11" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3307,11 +3306,11 @@
       </c>
       <c r="M12">
         <f t="shared" ca="1" si="0"/>
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="N12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.536986301369863</v>
+        <v>1.5232876712328767</v>
       </c>
       <c r="O12" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3324,7 +3323,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -3363,11 +3362,11 @@
       </c>
       <c r="M13">
         <f t="shared" ca="1" si="0"/>
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="N13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.6986301369863013</v>
+        <v>1.6849315068493151</v>
       </c>
       <c r="O13" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3410,11 +3409,11 @@
       </c>
       <c r="M14">
         <f t="shared" ca="1" si="0"/>
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="N14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.7835616438356163</v>
+        <v>1.7698630136986302</v>
       </c>
       <c r="O14" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3427,7 +3426,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="15" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -3466,11 +3465,11 @@
       </c>
       <c r="M15">
         <f t="shared" ca="1" si="0"/>
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="N15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>1.904109589041096</v>
+        <v>1.8904109589041096</v>
       </c>
       <c r="O15" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3513,11 +3512,11 @@
       </c>
       <c r="M16">
         <f t="shared" ca="1" si="0"/>
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="N16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2.032876712328767</v>
+        <v>2.0191780821917806</v>
       </c>
       <c r="O16" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3530,7 +3529,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -3569,11 +3568,11 @@
       </c>
       <c r="M17">
         <f t="shared" ca="1" si="0"/>
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="N17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2.2027397260273971</v>
+        <v>2.1890410958904107</v>
       </c>
       <c r="O17" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3616,11 +3615,11 @@
       </c>
       <c r="M18">
         <f t="shared" ca="1" si="0"/>
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="N18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2.536986301369863</v>
+        <v>2.5232876712328767</v>
       </c>
       <c r="O18" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3633,7 +3632,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -3672,11 +3671,11 @@
       </c>
       <c r="M19">
         <f t="shared" ca="1" si="0"/>
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="N19" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>2.7013698630136984</v>
+        <v>2.6876712328767125</v>
       </c>
       <c r="O19" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3719,11 +3718,11 @@
       </c>
       <c r="M20">
         <f t="shared" ca="1" si="0"/>
-        <v>1108</v>
+        <v>1103</v>
       </c>
       <c r="N20" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.0356164383561643</v>
+        <v>3.021917808219178</v>
       </c>
       <c r="O20" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3736,7 +3735,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -3775,11 +3774,11 @@
       </c>
       <c r="M21">
         <f t="shared" ca="1" si="0"/>
-        <v>1153</v>
+        <v>1148</v>
       </c>
       <c r="N21" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.1589041095890411</v>
+        <v>3.1452054794520548</v>
       </c>
       <c r="O21" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3789,7 +3788,7 @@
         <v>4370.9806120000003</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -3828,11 +3827,11 @@
       </c>
       <c r="M22">
         <f t="shared" ca="1" si="0"/>
-        <v>1170</v>
+        <v>1165</v>
       </c>
       <c r="N22" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.2054794520547945</v>
+        <v>3.1917808219178081</v>
       </c>
       <c r="O22" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3881,11 +3880,11 @@
       </c>
       <c r="M23">
         <f t="shared" ca="1" si="0"/>
-        <v>1292</v>
+        <v>1287</v>
       </c>
       <c r="N23" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.5397260273972604</v>
+        <v>3.526027397260274</v>
       </c>
       <c r="O23" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3931,11 +3930,11 @@
       </c>
       <c r="M24">
         <f t="shared" ca="1" si="0"/>
-        <v>1292</v>
+        <v>1287</v>
       </c>
       <c r="N24" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.5397260273972604</v>
+        <v>3.526027397260274</v>
       </c>
       <c r="O24" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -3948,7 +3947,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -3987,11 +3986,11 @@
       </c>
       <c r="M25">
         <f t="shared" ca="1" si="0"/>
-        <v>1351</v>
+        <v>1346</v>
       </c>
       <c r="N25" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.7013698630136984</v>
+        <v>3.6876712328767125</v>
       </c>
       <c r="O25" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4001,7 +4000,7 @@
         <v>16720.403074000002</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -4040,11 +4039,11 @@
       </c>
       <c r="M26">
         <f t="shared" ca="1" si="0"/>
-        <v>1426</v>
+        <v>1421</v>
       </c>
       <c r="N26" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>3.9068493150684933</v>
+        <v>3.893150684931507</v>
       </c>
       <c r="O26" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4054,7 +4053,7 @@
         <v>4302.1479799999997</v>
       </c>
     </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -4093,11 +4092,11 @@
       </c>
       <c r="M27">
         <f t="shared" ca="1" si="0"/>
-        <v>1535</v>
+        <v>1530</v>
       </c>
       <c r="N27" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4.2054794520547949</v>
+        <v>4.1917808219178081</v>
       </c>
       <c r="O27" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4140,11 +4139,11 @@
       </c>
       <c r="M28">
         <f t="shared" ca="1" si="0"/>
-        <v>1657</v>
+        <v>1652</v>
       </c>
       <c r="N28" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4.5397260273972604</v>
+        <v>4.5260273972602736</v>
       </c>
       <c r="O28" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4157,7 +4156,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -4196,11 +4195,11 @@
       </c>
       <c r="M29">
         <f t="shared" ca="1" si="0"/>
-        <v>1716</v>
+        <v>1711</v>
       </c>
       <c r="N29" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4.7013698630136984</v>
+        <v>4.6876712328767125</v>
       </c>
       <c r="O29" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4210,7 +4209,7 @@
         <v>16683.269703999998</v>
       </c>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -4249,11 +4248,11 @@
       </c>
       <c r="M30">
         <f t="shared" ca="1" si="0"/>
-        <v>1808</v>
+        <v>1803</v>
       </c>
       <c r="N30" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>4.9534246575342467</v>
+        <v>4.9397260273972599</v>
       </c>
       <c r="O30" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4263,7 +4262,7 @@
         <v>16678.621740999999</v>
       </c>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -4302,11 +4301,11 @@
       </c>
       <c r="M31">
         <f t="shared" ca="1" si="0"/>
-        <v>1883</v>
+        <v>1878</v>
       </c>
       <c r="N31" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.1589041095890407</v>
+        <v>5.1452054794520548</v>
       </c>
       <c r="O31" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4316,7 +4315,7 @@
         <v>4323.1214110000001</v>
       </c>
     </row>
-    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -4355,11 +4354,11 @@
       </c>
       <c r="M32">
         <f t="shared" ca="1" si="0"/>
-        <v>1900</v>
+        <v>1895</v>
       </c>
       <c r="N32" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.2054794520547949</v>
+        <v>5.1917808219178081</v>
       </c>
       <c r="O32" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4369,7 +4368,7 @@
         <v>16675.987335000002</v>
       </c>
     </row>
-    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -4408,11 +4407,11 @@
       </c>
       <c r="M33">
         <f t="shared" ca="1" si="0"/>
-        <v>1991</v>
+        <v>1986</v>
       </c>
       <c r="N33" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.4547945205479449</v>
+        <v>5.441095890410959</v>
       </c>
       <c r="O33" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4422,7 +4421,7 @@
         <v>16681.994450999999</v>
       </c>
     </row>
-    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -4461,11 +4460,11 @@
       </c>
       <c r="M34">
         <f t="shared" ca="1" si="0"/>
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="N34" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.5397260273972604</v>
+        <v>5.5260273972602736</v>
       </c>
       <c r="O34" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4514,11 +4513,11 @@
       </c>
       <c r="M35">
         <f t="shared" ca="1" si="0"/>
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="N35" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.5397260273972604</v>
+        <v>5.5260273972602736</v>
       </c>
       <c r="O35" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4531,7 +4530,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>21</v>
       </c>
@@ -4570,11 +4569,11 @@
       </c>
       <c r="M36">
         <f t="shared" ca="1" si="0"/>
-        <v>2081</v>
+        <v>2076</v>
       </c>
       <c r="N36" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.7013698630136984</v>
+        <v>5.6876712328767125</v>
       </c>
       <c r="O36" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4584,7 +4583,7 @@
         <v>16679.343266</v>
       </c>
     </row>
-    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -4623,11 +4622,11 @@
       </c>
       <c r="M37">
         <f t="shared" ca="1" si="0"/>
-        <v>2173</v>
+        <v>2168</v>
       </c>
       <c r="N37" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>5.9534246575342467</v>
+        <v>5.9397260273972599</v>
       </c>
       <c r="O37" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4670,11 +4669,11 @@
       </c>
       <c r="M38">
         <f t="shared" ca="1" si="0"/>
-        <v>2387</v>
+        <v>2382</v>
       </c>
       <c r="N38" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>6.5397260273972604</v>
+        <v>6.5260273972602736</v>
       </c>
       <c r="O38" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4687,7 +4686,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -4726,11 +4725,11 @@
       </c>
       <c r="M39">
         <f t="shared" ca="1" si="0"/>
-        <v>2614</v>
+        <v>2609</v>
       </c>
       <c r="N39" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>7.161643835616438</v>
+        <v>7.1479452054794521</v>
       </c>
       <c r="O39" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4779,11 +4778,11 @@
       </c>
       <c r="M40">
         <f t="shared" ca="1" si="0"/>
-        <v>2753</v>
+        <v>2748</v>
       </c>
       <c r="N40" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>7.5424657534246577</v>
+        <v>7.5287671232876709</v>
       </c>
       <c r="O40" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4796,7 +4795,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="41" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -4835,11 +4834,11 @@
       </c>
       <c r="M41">
         <f t="shared" ca="1" si="0"/>
-        <v>2887</v>
+        <v>2882</v>
       </c>
       <c r="N41" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>7.9095890410958907</v>
+        <v>7.8958904109589039</v>
       </c>
       <c r="O41" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4888,11 +4887,11 @@
       </c>
       <c r="M42">
         <f t="shared" ca="1" si="0"/>
-        <v>3483</v>
+        <v>3478</v>
       </c>
       <c r="N42" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>9.5424657534246577</v>
+        <v>9.5287671232876718</v>
       </c>
       <c r="O42" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4905,7 +4904,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>11</v>
       </c>
@@ -4944,11 +4943,11 @@
       </c>
       <c r="M43">
         <f t="shared" ca="1" si="0"/>
-        <v>3617</v>
+        <v>3612</v>
       </c>
       <c r="N43" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>9.9095890410958898</v>
+        <v>9.8958904109589039</v>
       </c>
       <c r="O43" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -4958,7 +4957,7 @@
         <v>4145.819074</v>
       </c>
     </row>
-    <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -4997,11 +4996,11 @@
       </c>
       <c r="M44">
         <f t="shared" ca="1" si="0"/>
-        <v>5536</v>
+        <v>5531</v>
       </c>
       <c r="N44" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>15.167123287671233</v>
+        <v>15.153424657534247</v>
       </c>
       <c r="O44" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -5011,7 +5010,7 @@
         <v>4156.0300610000004</v>
       </c>
     </row>
-    <row r="45" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>11</v>
       </c>
@@ -5050,11 +5049,11 @@
       </c>
       <c r="M45">
         <f t="shared" ca="1" si="0"/>
-        <v>7270</v>
+        <v>7265</v>
       </c>
       <c r="N45" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>19.917808219178081</v>
+        <v>19.904109589041095</v>
       </c>
       <c r="O45" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -5064,7 +5063,7 @@
         <v>4036.7481910000001</v>
       </c>
     </row>
-    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>11</v>
       </c>
@@ -5103,11 +5102,11 @@
       </c>
       <c r="M46">
         <f t="shared" ca="1" si="0"/>
-        <v>9188</v>
+        <v>9183</v>
       </c>
       <c r="N46" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>25.172602739726027</v>
+        <v>25.158904109589042</v>
       </c>
       <c r="O46" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -5117,7 +5116,7 @@
         <v>4067.5167569999999</v>
       </c>
     </row>
-    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>11</v>
       </c>
@@ -5156,11 +5155,11 @@
       </c>
       <c r="M47">
         <f t="shared" ca="1" si="0"/>
-        <v>10922</v>
+        <v>10917</v>
       </c>
       <c r="N47" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>29.923287671232877</v>
+        <v>29.909589041095892</v>
       </c>
       <c r="O47" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -5170,7 +5169,7 @@
         <v>3988.048245</v>
       </c>
     </row>
-    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>11</v>
       </c>
@@ -5209,11 +5208,11 @@
       </c>
       <c r="M48">
         <f t="shared" ca="1" si="0"/>
-        <v>12841</v>
+        <v>12836</v>
       </c>
       <c r="N48" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>35.180821917808217</v>
+        <v>35.167123287671231</v>
       </c>
       <c r="O48" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -5223,7 +5222,7 @@
         <v>4019.0382979999999</v>
       </c>
     </row>
-    <row r="49" spans="11:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="11:15" x14ac:dyDescent="0.25">
       <c r="L49" t="str">
         <f>MID(B49,7,4)</f>
         <v/>
@@ -5239,14 +5238,7 @@
       <c r="K58" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L49" xr:uid="{A970A97D-4899-4477-842A-DD8D42C7E015}">
-    <filterColumn colId="11">
-      <filters>
-        <filter val="LTN"/>
-        <filter val="NTNF"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L49" xr:uid="{A970A97D-4899-4477-842A-DD8D42C7E015}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K48">
     <sortCondition ref="D2:D48"/>
   </sortState>

</xml_diff>